<commit_message>
Link the companion set Greek Cities of Central and South Asia
The scope note and the README now link the new set 26 page, and the
left-out entries for Kandahar, Farah, Herat, Merv, Nisa, Achaia, Soteira
and the Sakastane towns no longer call it "in preparation". The cities,
counts and cards are unchanged (176 cities, 269 left out).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WtrLmt44Z4oEuT8DvyyCJq
</commit_message>
<xml_diff>
--- a/dl/greek-cities-west-asia.xlsx
+++ b/dl/greek-cities-west-asia.xlsx
@@ -11322,7 +11322,7 @@
     <t xml:space="preserve">Achaia/Achais</t>
   </si>
   <si>
-    <t xml:space="preserve">Seleucid foundation (Appian, Syr. 57; Strabo 11.10.1 places Achaia in Areia; Pliny 6.48 has Heraclea refounded as Achais), in present-day Afghanistan or Turkmenistan: counted in the companion set Greek Cities of Central and South Asia (in preparation).</t>
+    <t xml:space="preserve">Seleucid foundation (Appian, Syr. 57; Strabo 11.10.1 places Achaia in Areia; Pliny 6.48 has Heraclea refounded as Achais), in present-day Afghanistan or Turkmenistan: counted in the companion set Greek Cities of Central and South Asia.</t>
   </si>
   <si>
     <t xml:space="preserve">Shushtar (Tostar)</t>
@@ -11355,7 +11355,7 @@
     <t xml:space="preserve">Afghanistan</t>
   </si>
   <si>
-    <t xml:space="preserve">In present-day Afghanistan: counted in the companion set Greek Cities of Central and South Asia (in preparation).</t>
+    <t xml:space="preserve">In present-day Afghanistan: counted in the companion set Greek Cities of Central and South Asia.</t>
   </si>
   <si>
     <t xml:space="preserve">Prophthasia (Farah)</t>
@@ -11370,13 +11370,13 @@
     <t xml:space="preserve">Turkmenistan</t>
   </si>
   <si>
-    <t xml:space="preserve">In present-day Turkmenistan: counted in the companion set Greek Cities of Central and South Asia (in preparation).</t>
+    <t xml:space="preserve">In present-day Turkmenistan: counted in the companion set Greek Cities of Central and South Asia.</t>
   </si>
   <si>
     <t xml:space="preserve">Nisa (Mithradatkert)</t>
   </si>
   <si>
-    <t xml:space="preserve">In present-day Turkmenistan; the companion set Greek Cities of Central and South Asia (in preparation) leaves it out too: an Arsacid royal fortress, whose Greek art belongs to the court and whose documents are Parthian.</t>
+    <t xml:space="preserve">In present-day Turkmenistan; the companion set Greek Cities of Central and South Asia leaves it out too: an Arsacid royal fortress, whose Greek art belongs to the court and whose documents are Parthian.</t>
   </si>
   <si>
     <t xml:space="preserve">Eruandashat (Yervandashat)</t>
@@ -11631,7 +11631,7 @@
     <t xml:space="preserve">Alexandria and Alexandropolis in Sakastane</t>
   </si>
   <si>
-    <t xml:space="preserve">Named by Isidore of Charax (Parthian Stations 18) among the towns of Sakastane, which lies mostly in Afghanistan; nothing places them in Iranian Sistan. Alexandropolis is counted in the companion set Greek Cities of Central and South Asia (in preparation) (the Alexandria there is taken as a scribal repetition).</t>
+    <t xml:space="preserve">Named by Isidore of Charax (Parthian Stations 18) among the towns of Sakastane, which lies mostly in Afghanistan; nothing places them in Iranian Sistan. Alexandropolis is counted in the companion set Greek Cities of Central and South Asia (the Alexandria there is taken as a scribal repetition).</t>
   </si>
   <si>
     <t xml:space="preserve">Corada (Phoenice Libanensis)</t>
@@ -11814,7 +11814,7 @@
     <t xml:space="preserve">Soteira (Parthia)</t>
   </si>
   <si>
-    <t xml:space="preserve">Seleucus I's foundation in Parthia (Appian, Syr. 57); Ptolemy lists a Sotira in Areia, so it is counted in the companion set Greek Cities of Central and South Asia (in preparation).</t>
+    <t xml:space="preserve">Seleucus I's foundation in Parthia (Appian, Syr. 57); Ptolemy lists a Sotira in Areia, so it is counted in the companion set Greek Cities of Central and South Asia.</t>
   </si>
   <si>
     <t xml:space="preserve">Dahan-i Ghulaman (Zranka?)</t>

</xml_diff>